<commit_message>
feat: add silhouette, davies bouldin, and calinski harabasz score
</commit_message>
<xml_diff>
--- a/evaluation-result-indosbert.xlsx
+++ b/evaluation-result-indosbert.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,14 +444,14 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>threshold</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>embedding_model</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>metric</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>time</t>
@@ -499,25 +499,40 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>silhouette_score</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>davies_bouldin</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>calinski_harabasz</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>accuracy</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>precision</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>f1</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>intents</t>
         </is>
@@ -528,7 +543,7 @@
         <v>0.3</v>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="C2" t="n">
         <v>0.01</v>
@@ -539,256 +554,64 @@
       <c r="E2" t="n">
         <v>15</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>IndoSBERT</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>euclidean</t>
-        </is>
-      </c>
       <c r="H2" t="n">
-        <v>1.58</v>
+        <v>0.17</v>
       </c>
       <c r="I2" t="n">
-        <v>13.55</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="J2" t="n">
         <v>9</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L2" t="n">
-        <v>0.03</v>
+        <v>0.17</v>
       </c>
       <c r="M2" t="n">
-        <v>0.16</v>
+        <v>0.42</v>
       </c>
       <c r="N2" t="n">
-        <v>0.06</v>
+        <v>0.24</v>
       </c>
       <c r="O2" t="n">
-        <v>0.05</v>
+        <v>0.24</v>
       </c>
       <c r="P2" t="n">
-        <v>0.05</v>
+        <v>0.18</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.384508990318119</v>
+        <v>0.17</v>
       </c>
       <c r="R2" t="n">
-        <v>16.3</v>
+        <v>2.141</v>
       </c>
       <c r="S2" t="n">
-        <v>38.5</v>
+        <v>144.04</v>
       </c>
       <c r="T2" t="n">
-        <v>22.9</v>
+        <v>0.4674965421853389</v>
       </c>
       <c r="U2" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="V2" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="W2" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="X2" t="n">
         <v>2</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="B3" t="n">
-        <v>15</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>15</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>IndoSBERT</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="I3" t="n">
-        <v>86.31</v>
-      </c>
-      <c r="J3" t="n">
-        <v>38</v>
-      </c>
-      <c r="K3" t="n">
-        <v>11</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.5739972337482711</v>
-      </c>
-      <c r="R3" t="n">
-        <v>59.9</v>
-      </c>
-      <c r="S3" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="T3" t="n">
-        <v>56.00000000000001</v>
-      </c>
-      <c r="U3" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>15</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="n">
-        <v>15</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>IndoBERT</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>euclidean</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="I4" t="n">
-        <v>13.55</v>
-      </c>
-      <c r="J4" t="n">
-        <v>9</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.3858921161825726</v>
-      </c>
-      <c r="R4" t="n">
-        <v>18</v>
-      </c>
-      <c r="S4" t="n">
-        <v>38.6</v>
-      </c>
-      <c r="T4" t="n">
-        <v>24.4</v>
-      </c>
-      <c r="U4" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="B5" t="n">
-        <v>15</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>15</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>IndoBERT</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="I5" t="n">
-        <v>91.42</v>
-      </c>
-      <c r="J5" t="n">
-        <v>27</v>
-      </c>
-      <c r="K5" t="n">
-        <v>14</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.5034578146611342</v>
-      </c>
-      <c r="R5" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="S5" t="n">
-        <v>50.3</v>
-      </c>
-      <c r="T5" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="U5" t="n">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add fit predict with evaluate
</commit_message>
<xml_diff>
--- a/evaluation-result-indosbert.xlsx
+++ b/evaluation-result-indosbert.xlsx
@@ -419,12 +419,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>distance</t>
+          <t>initial_distance</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>minimum_samples</t>
+          <t>initial_minimum_samples</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.17</v>
+        <v>0.31</v>
       </c>
       <c r="I2" t="n">
         <v>70.40000000000001</v>

</xml_diff>